<commit_message>
ITTKI Nazorat: role permissions, empty expected-benefit field, E9 default 1 000 000
- Only Loyiha rahbari saves assessments and stage changes; only Buxgalter
  saves costs, imports, impairment, settings and runs reports; Ichki auditor
  is view-only. Refusals show an Uzbek message and are written to the audit
  log (action 'denied'). Rules in ittki/db/permissions.py.
- 'Kutilayotgan sof iqtisodiy naf' left empty stays empty (no '0'
  placeholder); 0 is stored only when typed explicitly.
- E9 threshold default 1 000 000 so'm; old databases still on the former
  default 0 are upgraded once, with an audit record, unless a user set 0.
- tests/test_permissions.py (39 tests); engine and existing tests unchanged.
- User manual sections 3, 6.1, 7, 9 and screenshots updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PGM9yVgDDA2vF5dBJ6fVfY
</commit_message>
<xml_diff>
--- a/ITTKI_Nazorat/docs/samples/amortizatsiya_jadvali.xlsx
+++ b/ITTKI_Nazorat/docs/samples/amortizatsiya_jadvali.xlsx
@@ -513,7 +513,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Tuzilgan: 11.10.2026 16:41 · ITTKI Nazorat</t>
+          <t>Tuzilgan: 12.10.2026 05:41 · ITTKI Nazorat</t>
         </is>
       </c>
     </row>
@@ -679,7 +679,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Tuzilgan: 11.10.2026 16:41 · ITTKI Nazorat</t>
+          <t>Tuzilgan: 12.10.2026 05:41 · ITTKI Nazorat</t>
         </is>
       </c>
     </row>

</xml_diff>